<commit_message>
fix(reporter-page): add export functionality
- add export functionality to reporter page

[Fixes ASP-1182]
</commit_message>
<xml_diff>
--- a/api/src/excelreports/reportTemplates/Reporters.xlsx
+++ b/api/src/excelreports/reportTemplates/Reporters.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22323"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5FDA5191-1E1D-43E2-B881-D3217756858E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{00B55CBC-FB46-42A7-8C52-4CB67D01BF5A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,7 +82,7 @@
     <t>&lt;confirmFollowUpRatio&gt;</t>
   </si>
   <si>
-    <t>&lt;acknowledgeRatio&gt;</t>
+    <t>&lt;acknowledgedRatio&gt;</t>
   </si>
   <si>
     <t>&lt;totalFlagged&gt;</t>

</xml_diff>

<commit_message>
fix(reporter): fix reporter list
- fix last seen date
- fix reporter template

[Fixes ASP-1220]
</commit_message>
<xml_diff>
--- a/api/src/excelreports/reportTemplates/Reporters.xlsx
+++ b/api/src/excelreports/reportTemplates/Reporters.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22323"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22413"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{00B55CBC-FB46-42A7-8C52-4CB67D01BF5A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{282D653E-E433-4FE5-AAEE-3DD84ED8FF4E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,9 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -23,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Aspect Reporters</t>
   </si>
@@ -52,6 +54,9 @@
     <t>Delivered</t>
   </si>
   <si>
+    <t>Requires Follow-up</t>
+  </si>
+  <si>
     <t>% Confirmed Follow-Up</t>
   </si>
   <si>
@@ -77,6 +82,9 @@
   </si>
   <si>
     <t>&lt;delivered&gt;</t>
+  </si>
+  <si>
+    <t>&lt;requiresFollowUp&gt;</t>
   </si>
   <si>
     <t>&lt;confirmFollowUpRatio&gt;</t>
@@ -123,7 +131,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -146,16 +154,49 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -470,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.85546875" style="1" customWidth="1"/>
@@ -478,19 +519,20 @@
     <col min="3" max="3" width="21.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="14" style="1" customWidth="1"/>
     <col min="5" max="5" width="20.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="23.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="20.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="19.140625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="6" width="20.42578125" style="6" customWidth="1"/>
+    <col min="7" max="7" width="23.7109375" style="9" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" style="9" customWidth="1"/>
+    <col min="9" max="9" width="19.140625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -498,67 +540,73 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" s="3" customFormat="1" ht="14.25">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:10" s="2" customFormat="1" ht="14.25">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="J4" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="2" t="s">
+    <row r="5" spans="1:10">
+      <c r="A5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="C5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="D5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="E5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="F5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="G5" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="H5" s="11" t="s">
         <v>21</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(reporter-page): modify excel file
- modify excel file

[Fixes ASP-1164]
</commit_message>
<xml_diff>
--- a/api/src/excelreports/reportTemplates/Reporters.xlsx
+++ b/api/src/excelreports/reportTemplates/Reporters.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22413"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{282D653E-E433-4FE5-AAEE-3DD84ED8FF4E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028" calcCompleted="0"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -63,9 +62,6 @@
     <t>% Acknowledge</t>
   </si>
   <si>
-    <t>Flagged</t>
-  </si>
-  <si>
     <t>Revoked</t>
   </si>
   <si>
@@ -93,17 +89,20 @@
     <t>&lt;acknowledgedRatio&gt;</t>
   </si>
   <si>
-    <t>&lt;totalFlagged&gt;</t>
-  </si>
-  <si>
     <t>&lt;revoked&gt;</t>
+  </si>
+  <si>
+    <t>On Treatment</t>
+  </si>
+  <si>
+    <t>&lt;onTreatment&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -257,7 +256,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -309,7 +308,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -503,16 +502,16 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="22.85546875" style="1" customWidth="1"/>
@@ -527,12 +526,12 @@
     <col min="11" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -540,12 +539,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="2" customFormat="1" ht="14.25">
+    <row r="4" spans="1:10" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -571,42 +570,42 @@
         <v>11</v>
       </c>
       <c r="I4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="5" t="s">
+      <c r="B5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="H5" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>21</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>